<commit_message>
Kalkulationstool: Volltest-Datei auf V2.12 (Land, Abschreibung, Miete, Restbuchwert), Tests und Vergleichsrechnung aktualisiert
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016ur4TFdB9RxEnSHrWfTJdJ
</commit_message>
<xml_diff>
--- a/Kalkulationstool/vergleich/Excel-Vorlage_mit_Testwerten.xlsx
+++ b/Kalkulationstool/vergleich/Excel-Vorlage_mit_Testwerten.xlsx
@@ -100,7 +100,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="279">
   <si>
     <t xml:space="preserve">Kalkulationstool Light</t>
   </si>
@@ -614,7 +614,13 @@
     <t xml:space="preserve">Staplerleasing</t>
   </si>
   <si>
+    <t xml:space="preserve">Regalerweiterung Halle 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Energie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Flurförderzeuge Mietpool</t>
   </si>
   <si>
     <t xml:space="preserve">Summe</t>
@@ -9155,19 +9161,25 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="192"/>
-      <c r="C7" s="193"/>
-      <c r="D7" s="194"/>
+      <c r="B7" s="192" t="s">
+        <v>166</v>
+      </c>
+      <c r="C7" s="193" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="194" t="n">
+        <v>240000</v>
+      </c>
       <c r="E7" s="195" t="n">
         <f aca="false">F7/'A. Start'!$E$5*12</f>
-        <v>0</v>
+        <v>48000</v>
       </c>
       <c r="F7" s="195" t="n">
         <f aca="false">C7*D7</f>
-        <v>0</v>
+        <v>240000</v>
       </c>
       <c r="H7" s="192" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I7" s="193" t="n">
         <v>1</v>
@@ -9196,16 +9208,22 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="192"/>
-      <c r="C8" s="193"/>
-      <c r="D8" s="194"/>
+      <c r="B8" s="192" t="s">
+        <v>168</v>
+      </c>
+      <c r="C8" s="193" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="194" t="n">
+        <v>36000</v>
+      </c>
       <c r="E8" s="195" t="n">
         <f aca="false">F8/'A. Start'!$E$5*12</f>
-        <v>0</v>
+        <v>14400</v>
       </c>
       <c r="F8" s="195" t="n">
         <f aca="false">C8*D8</f>
-        <v>0</v>
+        <v>72000</v>
       </c>
       <c r="H8" s="192"/>
       <c r="I8" s="193"/>
@@ -9617,20 +9635,20 @@
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="121" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C20" s="121"/>
       <c r="D20" s="121"/>
       <c r="E20" s="196" t="n">
         <f aca="false">SUM(E5:E19)</f>
-        <v>173481.2</v>
+        <v>235881.2</v>
       </c>
       <c r="F20" s="196" t="n">
         <f aca="false">SUM(F5:F19)</f>
-        <v>867406</v>
+        <v>1179406</v>
       </c>
       <c r="H20" s="121" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="I20" s="121"/>
       <c r="J20" s="121"/>
@@ -9643,7 +9661,7 @@
         <v>5703000</v>
       </c>
       <c r="N20" s="121" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="O20" s="121"/>
       <c r="P20" s="121"/>
@@ -9675,7 +9693,7 @@
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B22" s="199" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C22" s="135" t="n">
         <v>1</v>
@@ -10033,14 +10051,14 @@
   <sheetData>
     <row r="1" s="86" customFormat="true" ht="29.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B1" s="207" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C1" s="35" t="str">
         <f aca="false">_xlfn.TEXTJOIN(" / ",TRUE(),'A. Start'!B8,'A. Start'!B9)</f>
         <v>VIAS / LOG</v>
       </c>
       <c r="E1" s="208" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="F1" s="209" t="n">
         <f aca="false">'A. Start'!E8</f>
@@ -10107,7 +10125,7 @@
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="225" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C7" s="226" t="n">
         <f aca="false">'B. Basisdaten'!C8</f>
@@ -10125,7 +10143,7 @@
     </row>
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="230" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C8" s="231" t="n">
         <f aca="false">'B. Basisdaten'!C9</f>
@@ -10143,7 +10161,7 @@
     </row>
     <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="235" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C9" s="236" t="n">
         <f aca="false">'B. Basisdaten'!C10</f>
@@ -10161,10 +10179,10 @@
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E10" s="239" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F10" s="239" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G10" s="239" t="s">
         <v>124</v>
@@ -10172,14 +10190,14 @@
     </row>
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="240" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C11" s="241" t="n">
         <f aca="false">D30</f>
-        <v>3818013.24980544</v>
+        <v>3896572.98793965</v>
       </c>
       <c r="D11" s="242" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="E11" s="243" t="n">
         <f aca="false">'I-1. FTE-Gehälter'!C33</f>
@@ -10196,14 +10214,14 @@
     </row>
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="246" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C12" s="247" t="n">
         <f aca="false">E30</f>
-        <v>19090066.2490272</v>
+        <v>19482864.9396982</v>
       </c>
       <c r="D12" s="248" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="E12" s="249" t="n">
         <f aca="false">'I-2. FTE-Löhne'!C33</f>
@@ -10220,14 +10238,14 @@
     </row>
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="252" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C13" s="253" t="n">
         <f aca="false">C11/E13</f>
-        <v>168472.730272717</v>
+        <v>171939.238298495</v>
       </c>
       <c r="D13" s="254" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="E13" s="255" t="n">
         <f aca="false">E12+E11</f>
@@ -10244,19 +10262,19 @@
     </row>
     <row r="16" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="90" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C16" s="258" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D16" s="258" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E16" s="258" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F16" s="258" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10266,7 +10284,7 @@
       </c>
       <c r="C17" s="260" t="n">
         <f aca="false">E17/$E$25</f>
-        <v>0.130205949725555</v>
+        <v>0.127580836492564</v>
       </c>
       <c r="D17" s="139" t="n">
         <f aca="false">'I-1. FTE-Gehälter'!AG33</f>
@@ -10291,7 +10309,7 @@
       </c>
       <c r="C18" s="260" t="n">
         <f aca="false">E18/$E$25</f>
-        <v>0.344826177188372</v>
+        <v>0.337874054318973</v>
       </c>
       <c r="D18" s="139" t="n">
         <f aca="false">'I-2. FTE-Löhne'!AG33</f>
@@ -10316,19 +10334,19 @@
       </c>
       <c r="C19" s="260" t="n">
         <f aca="false">E19/$E$25</f>
-        <v>0.0514232213641677</v>
+        <v>0.0685101322299385</v>
       </c>
       <c r="D19" s="139" t="n">
         <f aca="false">'II. Sachkosten'!E20</f>
-        <v>173481.2</v>
+        <v>235881.2</v>
       </c>
       <c r="E19" s="139" t="n">
         <f aca="false">'II. Sachkosten'!F20</f>
-        <v>867406</v>
+        <v>1179406</v>
       </c>
       <c r="F19" s="139" t="n">
         <f aca="false">D19/$G$13</f>
-        <v>3.9844410133799</v>
+        <v>5.41761716869186</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -10338,7 +10356,7 @@
       </c>
       <c r="C20" s="260" t="n">
         <f aca="false">E20/$E$25</f>
-        <v>0.338096152712627</v>
+        <v>0.331279715473161</v>
       </c>
       <c r="D20" s="139" t="n">
         <f aca="false">'II. Sachkosten'!K20</f>
@@ -10360,7 +10378,7 @@
       </c>
       <c r="C21" s="260" t="n">
         <f aca="false">E21/$E$25</f>
-        <v>0.028456277976865</v>
+        <v>0.0278825641639694</v>
       </c>
       <c r="D21" s="139" t="n">
         <f aca="false">'II. Sachkosten'!Q20</f>
@@ -10382,7 +10400,7 @@
       </c>
       <c r="C22" s="260" t="n">
         <f aca="false">E22/$E$25</f>
-        <v>0.0059283912451802</v>
+        <v>0.00580886753416029</v>
       </c>
       <c r="D22" s="139" t="n">
         <f aca="false">'II. Sachkosten'!E22</f>
@@ -10399,7 +10417,7 @@
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B23" s="263" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C23" s="264" t="n">
         <f aca="false">E23/$E$25</f>
@@ -10407,15 +10425,15 @@
       </c>
       <c r="D23" s="265" t="n">
         <f aca="false">SUM(D17:D22)</f>
-        <v>3032647.92432046</v>
+        <v>3095047.92432046</v>
       </c>
       <c r="E23" s="265" t="n">
         <f aca="false">SUM(E17:E22)</f>
-        <v>15163239.6216023</v>
+        <v>15475239.6216023</v>
       </c>
       <c r="F23" s="266" t="n">
         <f aca="false">D23/$G$13</f>
-        <v>69.6525431505192</v>
+        <v>71.0857193058312</v>
       </c>
       <c r="G23" s="267"/>
       <c r="H23" s="267"/>
@@ -10426,7 +10444,7 @@
         <v>0.095</v>
       </c>
       <c r="B24" s="268" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C24" s="260" t="n">
         <f aca="false">E24/$E$25</f>
@@ -10434,15 +10452,15 @@
       </c>
       <c r="D24" s="139" t="n">
         <f aca="false">(D23/(1-$F$7-$F$8-SUM($C$7:$C$9))*SUM($C$7:$C$9))</f>
-        <v>340948.583207626</v>
+        <v>347963.96782301</v>
       </c>
       <c r="E24" s="139" t="n">
         <f aca="false">(E23/(1-$F$7-$F$8-SUM($C$7:$C$9))*SUM($C$7:$C$9))</f>
-        <v>1704742.91603813</v>
+        <v>1739819.83911505</v>
       </c>
       <c r="F24" s="137" t="n">
         <f aca="false">D24/$G$13</f>
-        <v>7.83075928911163</v>
+        <v>7.99188560243073</v>
       </c>
       <c r="G24" s="261" t="n">
         <v>2665898.50295564</v>
@@ -10450,7 +10468,7 @@
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B25" s="263" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C25" s="264" t="n">
         <f aca="false">E25/$E$25</f>
@@ -10458,15 +10476,15 @@
       </c>
       <c r="D25" s="265" t="n">
         <f aca="false">D23+D24</f>
-        <v>3373596.50752809</v>
+        <v>3443011.89214347</v>
       </c>
       <c r="E25" s="265" t="n">
         <f aca="false">E23+E24</f>
-        <v>16867982.5376404</v>
+        <v>17215059.4607174</v>
       </c>
       <c r="F25" s="266" t="n">
         <f aca="false">D25/$G$13</f>
-        <v>77.4833024396309</v>
+        <v>79.0776049082619</v>
       </c>
       <c r="G25" s="261"/>
     </row>
@@ -10480,15 +10498,15 @@
       </c>
       <c r="D26" s="139" t="n">
         <f aca="false">(D23/(1-$F$7-$F$8-SUM($C$7:$C$9))*$F$7)</f>
-        <v>179446.622740856</v>
+        <v>183138.930433163</v>
       </c>
       <c r="E26" s="139" t="n">
         <f aca="false">(E23/(1-$F$7-$F$8-SUM($C$7:$C$9))*$F$7)</f>
-        <v>897233.113704278</v>
+        <v>915694.652165817</v>
       </c>
       <c r="F26" s="137" t="n">
         <f aca="false">D26/$G$13</f>
-        <v>4.12145225742717</v>
+        <v>4.2062555802267</v>
       </c>
       <c r="G26" s="261" t="n">
         <v>1599539.10177338</v>
@@ -10496,7 +10514,7 @@
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B27" s="268" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C27" s="260" t="n">
         <f aca="false">E27/$E$28</f>
@@ -10504,15 +10522,15 @@
       </c>
       <c r="D27" s="139" t="n">
         <f aca="false">(D23/(1-$F$7-$F$8-SUM($C$7:$C$9))*$F$8)</f>
-        <v>35889.3245481711</v>
+        <v>36627.7860866327</v>
       </c>
       <c r="E27" s="139" t="n">
         <f aca="false">(E23/(1-$F$7-$F$8-SUM($C$7:$C$9))*$F$8)</f>
-        <v>179446.622740856</v>
+        <v>183138.930433163</v>
       </c>
       <c r="F27" s="137" t="n">
         <f aca="false">D27/$G$13</f>
-        <v>0.824290451485435</v>
+        <v>0.84125111604534</v>
       </c>
       <c r="G27" s="261" t="n">
         <v>533179.700591127</v>
@@ -10520,7 +10538,7 @@
     </row>
     <row r="28" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B28" s="90" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C28" s="269" t="n">
         <f aca="false">E28/$E$25</f>
@@ -10528,15 +10546,15 @@
       </c>
       <c r="D28" s="270" t="n">
         <f aca="false">D25+D26+D27</f>
-        <v>3588932.45481711</v>
+        <v>3662778.60866327</v>
       </c>
       <c r="E28" s="270" t="n">
         <f aca="false">E25+E26+E27</f>
-        <v>17944662.2740856</v>
+        <v>18313893.0433163</v>
       </c>
       <c r="F28" s="271" t="n">
         <f aca="false">D28/$G$13</f>
-        <v>82.4290451485435</v>
+        <v>84.125111604534</v>
       </c>
       <c r="G28" s="261" t="n">
         <v>26658985.0295564</v>
@@ -10544,7 +10562,7 @@
     </row>
     <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B29" s="268" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C29" s="260" t="n">
         <f aca="false">E29/$E$30</f>
@@ -10552,15 +10570,15 @@
       </c>
       <c r="D29" s="139" t="n">
         <f aca="false">$F$9*((D23/(1-$F$7-$F$8-SUM($C$7:$C$9))))/(1-$F$9)</f>
-        <v>229080.794988326</v>
+        <v>233794.379276379</v>
       </c>
       <c r="E29" s="139" t="n">
         <f aca="false">$F$9*((E23/(1-$F$7-$F$8-SUM($C$7:$C$9))))/(1-$F$9)</f>
-        <v>1145403.97494163</v>
+        <v>1168971.89638189</v>
       </c>
       <c r="F29" s="137" t="n">
         <f aca="false">D29/$G$13</f>
-        <v>5.26142841373682</v>
+        <v>5.36968797475749</v>
       </c>
       <c r="G29" s="261" t="n">
         <v>2318172.61126577</v>
@@ -10568,7 +10586,7 @@
     </row>
     <row r="30" customFormat="false" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B30" s="90" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C30" s="272" t="n">
         <f aca="false">E30/E25</f>
@@ -10576,48 +10594,48 @@
       </c>
       <c r="D30" s="270" t="n">
         <f aca="false">D28+D29</f>
-        <v>3818013.24980544</v>
+        <v>3896572.98793965</v>
       </c>
       <c r="E30" s="270" t="n">
         <f aca="false">E28+E29</f>
-        <v>19090066.2490272</v>
+        <v>19482864.9396982</v>
       </c>
       <c r="F30" s="271" t="n">
         <f aca="false">D30/$G$13</f>
-        <v>87.6904735622803</v>
+        <v>89.4947995792915</v>
       </c>
       <c r="G30" s="261" t="n">
         <v>28977157.6408221</v>
       </c>
       <c r="H30" s="182" t="n">
         <f aca="false">E30/G30-1</f>
-        <v>-0.34120294041077</v>
+        <v>-0.327647480778054</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="49" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C32" s="88" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D32" s="88" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="94" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C33" s="273"/>
       <c r="D33" s="274" t="n">
         <f aca="false">D30</f>
-        <v>3818013.24980544</v>
+        <v>3896572.98793965</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="94" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C34" s="275" t="n">
         <f aca="false">D34/D33</f>
@@ -10625,12 +10643,12 @@
       </c>
       <c r="D34" s="276" t="n">
         <f aca="false">D26+D29</f>
-        <v>408527.417729182</v>
+        <v>416933.309709542</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="94" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C35" s="277" t="n">
         <f aca="false">C34+C7+C8</f>
@@ -10638,27 +10656,27 @@
       </c>
       <c r="D35" s="276" t="n">
         <f aca="false">C35*D33</f>
-        <v>694878.41146459</v>
+        <v>709176.283805016</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="49" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="94" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C38" s="273"/>
       <c r="D38" s="274" t="n">
         <f aca="false">D28</f>
-        <v>3588932.45481711</v>
+        <v>3662778.60866327</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="94" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C39" s="275" t="n">
         <f aca="false">D39/D38</f>
@@ -10666,12 +10684,12 @@
       </c>
       <c r="D39" s="276" t="n">
         <f aca="false">D26</f>
-        <v>179446.622740856</v>
+        <v>183138.930433163</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="94" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C40" s="277" t="n">
         <f aca="false">C39+C7+C8</f>
@@ -10679,7 +10697,7 @@
       </c>
       <c r="D40" s="276" t="n">
         <f aca="false">C40*D38</f>
-        <v>448616.556852139</v>
+        <v>457847.326082908</v>
       </c>
     </row>
   </sheetData>
@@ -10717,7 +10735,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="279" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="B1" s="279"/>
       <c r="C1" s="279"/>
@@ -10727,12 +10745,12 @@
       <c r="G1" s="279"/>
       <c r="H1" s="279"/>
       <c r="I1" s="280" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="J1" s="280"/>
       <c r="K1" s="280"/>
       <c r="L1" s="281" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="M1" s="281"/>
     </row>
@@ -10751,7 +10769,7 @@
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="282"/>
       <c r="B3" s="286" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="C3" s="286"/>
       <c r="D3" s="286"/>
@@ -10783,11 +10801,11 @@
     <row r="5" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="282"/>
       <c r="B5" s="287" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C5" s="288"/>
       <c r="D5" s="289" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="E5" s="290"/>
       <c r="F5" s="290"/>
@@ -10802,11 +10820,11 @@
     <row r="6" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="282"/>
       <c r="B6" s="291" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C6" s="291"/>
       <c r="D6" s="292" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E6" s="290"/>
       <c r="F6" s="290"/>
@@ -10821,7 +10839,7 @@
     <row r="7" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="282"/>
       <c r="B7" s="287" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D7" s="293" t="str">
         <f aca="false">'A. Start'!B8</f>
@@ -10836,7 +10854,7 @@
     <row r="8" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="282"/>
       <c r="B8" s="294" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D8" s="295"/>
       <c r="E8" s="295"/>
@@ -10844,13 +10862,13 @@
       <c r="G8" s="295"/>
       <c r="H8" s="296"/>
       <c r="I8" s="297" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="282"/>
       <c r="B9" s="287" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D9" s="298" t="str">
         <f aca="false">'A. Start'!B4</f>
@@ -10865,7 +10883,7 @@
     <row r="10" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="282"/>
       <c r="B10" s="287" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D10" s="298" t="str">
         <f aca="false">'A. Start'!B3</f>
@@ -10880,7 +10898,7 @@
     <row r="11" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="282"/>
       <c r="B11" s="287" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D11" s="298" t="str">
         <f aca="false">'A. Start'!E9</f>
@@ -10895,7 +10913,7 @@
     <row r="12" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="282"/>
       <c r="B12" s="287" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D12" s="298" t="str">
         <f aca="false">'A. Start'!B9</f>
@@ -10910,7 +10928,7 @@
     <row r="13" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="282"/>
       <c r="B13" s="287" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D13" s="300"/>
       <c r="E13" s="300"/>
@@ -10922,11 +10940,11 @@
     <row r="14" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="282"/>
       <c r="B14" s="301" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="C14" s="302"/>
       <c r="D14" s="300" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E14" s="300"/>
       <c r="F14" s="300"/>
@@ -10937,7 +10955,7 @@
     <row r="15" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="282"/>
       <c r="B15" s="301" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C15" s="302"/>
       <c r="D15" s="303" t="n">
@@ -10950,7 +10968,7 @@
     </row>
     <row r="16" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B16" s="304" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="C16" s="304"/>
       <c r="D16" s="305" t="n">
@@ -10969,7 +10987,7 @@
     <row r="18" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="282"/>
       <c r="B18" s="306" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C18" s="307"/>
       <c r="D18" s="307"/>
@@ -10983,14 +11001,14 @@
       <c r="A19" s="282"/>
       <c r="B19" s="308" t="n">
         <f aca="false">'V. Summary'!D33</f>
-        <v>3818013.24980544</v>
+        <v>3896572.98793965</v>
       </c>
       <c r="C19" s="309" t="str">
         <f aca="false">D14</f>
         <v>EUR</v>
       </c>
       <c r="D19" s="310" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="E19" s="310"/>
       <c r="F19" s="310"/>
@@ -11002,11 +11020,11 @@
     <row r="20" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="282"/>
       <c r="B20" s="306" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="C20" s="313"/>
       <c r="D20" s="314" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="E20" s="314"/>
       <c r="G20" s="311"/>
@@ -11018,7 +11036,7 @@
       <c r="A21" s="282"/>
       <c r="B21" s="308" t="n">
         <f aca="false">'V. Summary'!D35</f>
-        <v>694878.41146459</v>
+        <v>709176.283805016</v>
       </c>
       <c r="C21" s="309" t="str">
         <f aca="false">C19</f>
@@ -11036,11 +11054,11 @@
     <row r="22" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="282"/>
       <c r="B22" s="317" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C22" s="318"/>
       <c r="D22" s="319" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="E22" s="319"/>
       <c r="F22" s="320"/>
@@ -11055,7 +11073,7 @@
       <c r="A23" s="282"/>
       <c r="B23" s="308" t="n">
         <f aca="false">'V. Summary'!D34</f>
-        <v>408527.417729182</v>
+        <v>416933.309709542</v>
       </c>
       <c r="C23" s="322" t="str">
         <f aca="false">C19</f>
@@ -11075,7 +11093,7 @@
     <row r="24" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="282"/>
       <c r="B24" s="317" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C24" s="318"/>
       <c r="F24" s="323"/>
@@ -11085,7 +11103,7 @@
       <c r="A25" s="282"/>
       <c r="B25" s="308" t="n">
         <f aca="false">'V. Summary'!E19</f>
-        <v>867406</v>
+        <v>1179406</v>
       </c>
       <c r="C25" s="309" t="str">
         <f aca="false">C19</f>
@@ -11098,7 +11116,7 @@
     <row r="26" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="282"/>
       <c r="B26" s="317" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C26" s="318"/>
       <c r="I26" s="297"/>
@@ -11123,7 +11141,7 @@
     <row r="28" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="282"/>
       <c r="B28" s="327" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="I28" s="297"/>
     </row>
@@ -11139,7 +11157,7 @@
     <row r="31" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="282"/>
       <c r="B31" s="329" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C31" s="330"/>
       <c r="D31" s="331"/>
@@ -11156,7 +11174,7 @@
     <row r="33" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="282"/>
       <c r="B33" s="286" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C33" s="286"/>
       <c r="D33" s="286"/>
@@ -11169,7 +11187,7 @@
     <row r="34" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="282"/>
       <c r="B34" s="332" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="I34" s="297"/>
     </row>
@@ -11177,7 +11195,7 @@
       <c r="A35" s="333"/>
       <c r="B35" s="334" t="n">
         <f aca="false">'V. Summary'!D38</f>
-        <v>3588932.45481711</v>
+        <v>3662778.60866327</v>
       </c>
       <c r="C35" s="309" t="str">
         <f aca="false">C19</f>
@@ -11189,10 +11207,10 @@
     <row r="36" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="333"/>
       <c r="B36" s="306" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D36" s="319" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I36" s="297"/>
       <c r="K36" s="312"/>
@@ -11201,7 +11219,7 @@
       <c r="A37" s="333"/>
       <c r="B37" s="335" t="n">
         <f aca="false">'V. Summary'!D40</f>
-        <v>448616.556852139</v>
+        <v>457847.326082908</v>
       </c>
       <c r="C37" s="309" t="str">
         <f aca="false">C35</f>
@@ -11217,10 +11235,10 @@
     <row r="38" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="333"/>
       <c r="B38" s="306" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D38" s="319" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="G38" s="321" t="n">
         <f aca="false">D37-D39</f>
@@ -11232,7 +11250,7 @@
     <row r="39" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="335" t="n">
         <f aca="false">'V. Summary'!D39</f>
-        <v>179446.622740856</v>
+        <v>183138.930433163</v>
       </c>
       <c r="C39" s="322" t="str">
         <f aca="false">C35</f>
@@ -11251,14 +11269,14 @@
     </row>
     <row r="40" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="306" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="I40" s="297"/>
     </row>
     <row r="41" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="335" t="n">
         <f aca="false">B25</f>
-        <v>867406</v>
+        <v>1179406</v>
       </c>
       <c r="C41" s="322" t="str">
         <f aca="false">C35</f>
@@ -11271,7 +11289,7 @@
     </row>
     <row r="42" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B42" s="306" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C42" s="318"/>
       <c r="F42" s="338"/>
@@ -11401,10 +11419,10 @@
   <sheetData>
     <row r="2" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="F2" s="0" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="G2" s="0" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11414,55 +11432,55 @@
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="0" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D4" s="342" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E4" s="343" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="M4" s="343" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="N4" s="343" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="O4" s="343" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="0" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D5" s="342"/>
       <c r="E5" s="343" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="G5" s="344" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="N5" s="343" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D6" s="342"/>
       <c r="E6" s="343" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="G6" s="344" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D7" s="342"/>
       <c r="E7" s="343" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="G7" s="343" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11470,15 +11488,15 @@
       <c r="E8" s="345"/>
       <c r="F8" s="345"/>
       <c r="G8" s="346" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D9" s="0" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F9" s="347" t="n">
         <v>0.238</v>
@@ -11489,12 +11507,12 @@
       <c r="E10" s="345"/>
       <c r="F10" s="345"/>
       <c r="G10" s="345" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E11" s="0" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F11" s="348"/>
       <c r="G11" s="348"/>
@@ -11508,17 +11526,17 @@
       <c r="E12" s="345"/>
       <c r="F12" s="345"/>
       <c r="G12" s="345" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D13" s="0" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11526,7 +11544,7 @@
       <c r="E15" s="345"/>
       <c r="F15" s="345"/>
       <c r="G15" s="345" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11536,7 +11554,7 @@
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D17" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11544,59 +11562,59 @@
       <c r="E18" s="345"/>
       <c r="F18" s="345"/>
       <c r="G18" s="345" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E19" s="343" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="G19" s="343" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D28" s="0" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F28" s="0" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="G28" s="0" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="H28" s="0" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="I28" s="343" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="J28" s="343" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="K28" s="343" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="L28" s="343" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="M28" s="343" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="O28" s="343" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="P28" s="343" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="Q28" s="343" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="S28" s="343" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>